<commit_message>
Update-in-place training log + local session-struct export
training_log.xlsx now updates in place (multi-box-safe: only touches the
subject sheet(s) found on this machine, matches rows by SESSION-STARTED,
never overwrites hand-typed Weight/Notes/header cells) instead of rebuilding
from scratch. Session-CSV parsing extracted to session_csv_parser.py, shared
with the new session_struct_export.py, which both task scripts now call at
every termination path (Kill, Stop, normal finish) to save a local .mat/.json
snapshot of everything needed to recreate that session.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt formatCode="0.0%" numFmtId="164"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -53,7 +55,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -61,6 +63,7 @@
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="0" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
@@ -426,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:X16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="14"/>
@@ -450,6 +453,9 @@
     <col customWidth="1" max="19" min="19" width="14"/>
     <col customWidth="1" max="20" min="20" width="14"/>
     <col customWidth="1" max="21" min="21" width="14"/>
+    <col customWidth="1" hidden="1" max="22" min="22" width="14"/>
+    <col customWidth="1" max="23" min="23" width="14"/>
+    <col customWidth="1" max="24" min="24" width="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,7 +471,11 @@
           <t>DOB</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -473,7 +483,6 @@
           <t>Sex</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -481,7 +490,6 @@
           <t>Strain</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -489,7 +497,6 @@
           <t>Baseline weight (g)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -597,9 +604,23 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>Session started</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="inlineStr">
+        <is>
+          <t>Session data (local path)</t>
+        </is>
+      </c>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>Session struct (local path)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>stage2_threshold_staircase</t>
@@ -626,7 +647,6 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -681,7 +701,6 @@
       <c r="P9" t="n">
         <v>2</v>
       </c>
-      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -736,7 +755,6 @@
       <c r="P10" t="n">
         <v>2</v>
       </c>
-      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -794,7 +812,6 @@
       <c r="R11" t="b">
         <v>0</v>
       </c>
-      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -852,7 +869,297 @@
       <c r="R12" t="b">
         <v>0</v>
       </c>
-      <c r="U12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>stage1_wheel_shaping</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" t="n">
+        <v>8.220500000000001</v>
+      </c>
+      <c r="E13" t="n">
+        <v>15</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" t="n">
+        <v>9</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.1000000000000001</v>
+      </c>
+      <c r="L13" t="n">
+        <v>7</v>
+      </c>
+      <c r="M13" t="n">
+        <v>7</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P13" t="n">
+        <v>2</v>
+      </c>
+      <c r="S13" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="T13" s="5">
+        <f>IFERROR(S13/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>handled by hand</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:41:46.605630</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134145\20260811-134145.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>stage1_wheel_shaping</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>125</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10.4758</v>
+      </c>
+      <c r="E14" t="n">
+        <v>123</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>95</v>
+      </c>
+      <c r="I14" t="n">
+        <v>29</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.09999999999999977</v>
+      </c>
+      <c r="L14" t="n">
+        <v>7</v>
+      </c>
+      <c r="M14" t="n">
+        <v>7</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P14" t="n">
+        <v>2</v>
+      </c>
+      <c r="T14" s="5">
+        <f>IFERROR(S14/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:46:30.773972</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134630\20260811-134630.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>stage2_threshold_staircase</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>68</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6.3955</v>
+      </c>
+      <c r="E15" t="n">
+        <v>68</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>40</v>
+      </c>
+      <c r="I15" t="n">
+        <v>28</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.09999999999999991</v>
+      </c>
+      <c r="L15" t="n">
+        <v>7</v>
+      </c>
+      <c r="M15" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="R15" t="b">
+        <v>0</v>
+      </c>
+      <c r="T15" s="5">
+        <f>IFERROR(S15/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:51:34.028274</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135132\20260811-135132.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>stage2_threshold_staircase</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>69</v>
+      </c>
+      <c r="D16" t="n">
+        <v>10.4654</v>
+      </c>
+      <c r="E16" t="n">
+        <v>34</v>
+      </c>
+      <c r="F16" t="n">
+        <v>9</v>
+      </c>
+      <c r="G16" t="n">
+        <v>26</v>
+      </c>
+      <c r="H16" t="n">
+        <v>29</v>
+      </c>
+      <c r="I16" t="n">
+        <v>14</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.1000000000000001</v>
+      </c>
+      <c r="L16" t="n">
+        <v>7</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="R16" t="b">
+        <v>0</v>
+      </c>
+      <c r="T16" s="5">
+        <f>IFERROR(S16/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:53:54.632954</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135354\20260811-135354.csv</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135354\20260811-135354_struct.mat</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>

</xml_diff>

<commit_message>
Canonicalize training-log column order every run, add merge-verify toggle
The table (header row included) is now fully cleared and rewritten in
COLUMNS' own canonical order every run, instead of only ever appending new
columns to whatever historical order a sheet already had -- that's why
Weight (g)/Weight % were stuck in their original positions despite the
schema listing them earlier. Dropped the 'Protocol / Stage' column
entirely (redundant with the section header each row already sits under);
Weight (g)/Weight % now land at C/D as a direct result.

Also confirmed the two new sessions that "didn't merge" were run under the
GUI's test subject again, same as before -- not a bug. Added
_MERGE_TEST_SUBJECT (default False) so this can be verified directly
against real bench data without waiting for a real animal session.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC19"/>
+  <dimension ref="A1:Z21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="14"/>
@@ -473,7 +473,7 @@
     <col customWidth="1" max="21" min="21" width="14"/>
     <col customWidth="1" hidden="1" max="22" min="22" width="14"/>
     <col customWidth="1" max="23" min="23" width="14"/>
-    <col customWidth="1" max="24" min="24" width="14"/>
+    <col customWidth="1" hidden="1" max="24" min="24" width="14"/>
     <col customWidth="1" max="25" min="25" width="14"/>
     <col customWidth="1" max="26" min="26" width="14"/>
     <col customWidth="1" max="27" min="27" width="14"/>
@@ -529,142 +529,127 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Protocol / Stage</t>
+          <t>Time (HH:MM)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>Weight (g)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Weight %</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>Trials</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Duration (s)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Rewards</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Reward Amount (uL)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Total Volume (uL)</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Aborts</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Withheld</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>No-movement</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>L turns</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>R turns</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>Licks</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Reward duration (s)</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>Threshold start (deg)</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>Threshold end (deg)</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>Threshold end (% final)</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>ITI (s)</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="S7" s="3" t="inlineStr">
         <is>
           <t>Gain mult (Stage 1)</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>Direction ratio (Stage 2)</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
+      <c r="U7" s="3" t="inlineStr">
         <is>
           <t>Simple gates met (Stage 2)</t>
         </is>
       </c>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>Weight (g)</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>Weight %</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>Num. Sessions</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="V7" s="3" t="inlineStr">
+      <c r="X7" s="3" t="inlineStr">
         <is>
           <t>Session started</t>
         </is>
       </c>
-      <c r="W7" s="3" t="inlineStr">
+      <c r="Y7" s="3" t="inlineStr">
         <is>
           <t>Session data (local path)</t>
         </is>
       </c>
-      <c r="X7" s="3" t="inlineStr">
+      <c r="Z7" s="3" t="inlineStr">
         <is>
           <t>Session struct (local path)</t>
-        </is>
-      </c>
-      <c r="Y7" s="3" t="inlineStr">
-        <is>
-          <t>Num. Sessions</t>
-        </is>
-      </c>
-      <c r="Z7" s="3" t="inlineStr">
-        <is>
-          <t>Reward Amount (uL)</t>
-        </is>
-      </c>
-      <c r="AA7" s="3" t="inlineStr">
-        <is>
-          <t>Total Volume (uL)</t>
-        </is>
-      </c>
-      <c r="AB7" s="3" t="inlineStr">
-        <is>
-          <t>Aborts</t>
-        </is>
-      </c>
-      <c r="AC7" s="3" t="inlineStr">
-        <is>
-          <t>Time (HH:MM)</t>
         </is>
       </c>
     </row>
@@ -699,9 +684,6 @@
       <c r="X8" s="7" t="n"/>
       <c r="Y8" s="7" t="n"/>
       <c r="Z8" s="7" t="n"/>
-      <c r="AA8" s="7" t="n"/>
-      <c r="AB8" s="7" t="n"/>
-      <c r="AC8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -711,76 +693,71 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>stage1_wheel_shaping</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="C9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D9" s="5">
+        <f>IFERROR(C9/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E9" t="n">
         <v>15</v>
       </c>
-      <c r="D9" t="n">
+      <c r="F9" t="n">
         <v>8.220500000000001</v>
       </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
         <v>6</v>
       </c>
-      <c r="I9" t="n">
+      <c r="M9" t="n">
         <v>9</v>
       </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
         <v>7</v>
       </c>
-      <c r="M9" t="n">
+      <c r="P9" t="n">
         <v>7</v>
       </c>
-      <c r="N9" s="4" t="n">
+      <c r="Q9" s="4" t="n">
         <v>0.2</v>
       </c>
-      <c r="O9" t="n">
+      <c r="R9" t="n">
         <v>0.5</v>
       </c>
-      <c r="P9" t="n">
+      <c r="S9" t="n">
         <v>2</v>
       </c>
-      <c r="S9" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="T9" s="5">
-        <f>IFERROR(S9/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="U9" t="inlineStr">
+      <c r="V9" t="n">
+        <v>1</v>
+      </c>
+      <c r="W9" t="inlineStr">
         <is>
           <t>handled by hand</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>2026-08-11 13:41:46.605630</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134145\20260811-134145.csv</t>
-        </is>
-      </c>
-      <c r="Y9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>13:41</t>
         </is>
       </c>
     </row>
@@ -792,68 +769,63 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>stage1_wheel_shaping</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
+          <t>13:46</t>
+        </is>
+      </c>
+      <c r="D10" s="5">
+        <f>IFERROR(C10/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E10" t="n">
         <v>125</v>
       </c>
-      <c r="D10" t="n">
+      <c r="F10" t="n">
         <v>10.4758</v>
       </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
         <v>2</v>
       </c>
-      <c r="H10" t="n">
+      <c r="L10" t="n">
         <v>95</v>
       </c>
-      <c r="I10" t="n">
+      <c r="M10" t="n">
         <v>29</v>
       </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
         <v>7</v>
       </c>
-      <c r="M10" t="n">
+      <c r="P10" t="n">
         <v>7</v>
       </c>
-      <c r="N10" s="4" t="n">
+      <c r="Q10" s="4" t="n">
         <v>0.2</v>
       </c>
-      <c r="O10" t="n">
+      <c r="R10" t="n">
         <v>0.5</v>
       </c>
-      <c r="P10" t="n">
+      <c r="S10" t="n">
         <v>2</v>
       </c>
-      <c r="T10" s="5">
-        <f>IFERROR(S10/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="V10" t="inlineStr">
+      <c r="V10" t="n">
+        <v>1</v>
+      </c>
+      <c r="X10" t="inlineStr">
         <is>
           <t>2026-08-11 13:46:30.773972</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134630\20260811-134630.csv</t>
-        </is>
-      </c>
-      <c r="Y10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>13:46</t>
         </is>
       </c>
     </row>
@@ -865,79 +837,74 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>stage1_wheel_shaping</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
+          <t>11:14</t>
+        </is>
+      </c>
+      <c r="D11" s="5">
+        <f>IFERROR(C11/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E11" t="n">
         <v>6</v>
       </c>
-      <c r="D11" t="n">
+      <c r="F11" t="n">
         <v>4.019900000000001</v>
       </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
         <v>3</v>
       </c>
-      <c r="I11" t="n">
+      <c r="M11" t="n">
         <v>3</v>
       </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
         <v>1.75</v>
       </c>
-      <c r="M11" t="n">
+      <c r="P11" t="n">
         <v>1.75</v>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="Q11" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="O11" t="n">
+      <c r="R11" t="n">
         <v>0.4999999999999999</v>
       </c>
-      <c r="P11" t="n">
+      <c r="S11" t="n">
         <v>2</v>
       </c>
-      <c r="T11" s="5">
-        <f>IFERROR(S11/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="V11" t="inlineStr">
+      <c r="V11" t="n">
+        <v>1</v>
+      </c>
+      <c r="X11" t="inlineStr">
         <is>
           <t>2026-08-13 11:14:02.776900</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-111402\20260813-111402.csv</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-111402\20260813-111402_struct.mat</t>
-        </is>
-      </c>
-      <c r="Y11" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>11:14</t>
         </is>
       </c>
     </row>
@@ -949,19 +916,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>stage1_wheel_shaping</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="D12" s="5">
+        <f>IFERROR(C12/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
@@ -970,29 +932,29 @@
       <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="T12" s="5">
-        <f>IFERROR(S12/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="V12" t="inlineStr">
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X12" t="inlineStr">
         <is>
           <t>2026-08-13 13:22:19.337954</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="Y12" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132218\20260813-132218.csv</t>
-        </is>
-      </c>
-      <c r="Y12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>13:22</t>
         </is>
       </c>
     </row>
@@ -1004,79 +966,74 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>stage1_wheel_shaping</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="D13" s="5">
+        <f>IFERROR(C13/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E13" t="n">
         <v>32</v>
       </c>
-      <c r="D13" t="n">
+      <c r="F13" t="n">
         <v>10.3488</v>
       </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
       <c r="G13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
         <v>6</v>
       </c>
-      <c r="H13" t="n">
+      <c r="L13" t="n">
         <v>17</v>
       </c>
-      <c r="I13" t="n">
+      <c r="M13" t="n">
         <v>9</v>
       </c>
-      <c r="J13" t="n">
+      <c r="N13" t="n">
         <v>17</v>
       </c>
-      <c r="L13" t="n">
+      <c r="O13" t="n">
         <v>1.75</v>
       </c>
-      <c r="M13" t="n">
+      <c r="P13" t="n">
         <v>1.75</v>
       </c>
-      <c r="N13" s="4" t="n">
+      <c r="Q13" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="O13" t="n">
+      <c r="R13" t="n">
         <v>0.5</v>
       </c>
-      <c r="P13" t="n">
+      <c r="S13" t="n">
         <v>2</v>
       </c>
-      <c r="T13" s="5">
-        <f>IFERROR(S13/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="V13" t="inlineStr">
+      <c r="V13" t="n">
+        <v>1</v>
+      </c>
+      <c r="X13" t="inlineStr">
         <is>
           <t>2026-08-13 13:29:35.160305</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132934\20260813-132934.csv</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132934\20260813-132934_struct.mat</t>
-        </is>
-      </c>
-      <c r="Y13" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB13" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>13:29</t>
         </is>
       </c>
     </row>
@@ -1088,396 +1045,523 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>stage1_wheel_shaping</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="D14" s="5">
+        <f>IFERROR(C14/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E14" t="n">
         <v>15</v>
       </c>
-      <c r="D14" t="n">
+      <c r="F14" t="n">
         <v>1.5698</v>
       </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
         <v>7</v>
       </c>
-      <c r="I14" t="n">
+      <c r="M14" t="n">
         <v>8</v>
       </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
         <v>1.75</v>
       </c>
-      <c r="M14" t="n">
+      <c r="P14" t="n">
         <v>1.75</v>
       </c>
-      <c r="N14" s="4" t="n">
+      <c r="Q14" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="O14" t="n">
+      <c r="R14" t="n">
         <v>0.5</v>
       </c>
-      <c r="P14" t="n">
+      <c r="S14" t="n">
         <v>2</v>
       </c>
-      <c r="T14" s="5">
-        <f>IFERROR(S14/$B$5,"")</f>
+      <c r="V14" t="n">
+        <v>1</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>2026-08-13 13:31:59.325021</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-133158\20260813-133158.csv</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-133158\20260813-133158_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="D15" s="5">
+        <f>IFERROR(C15/$B$5,"")</f>
         <v/>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>2026-08-13 13:31:59.325021</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-133158\20260813-133158.csv</t>
-        </is>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-133158\20260813-133158_struct.mat</t>
-        </is>
-      </c>
-      <c r="Y14" t="n">
+      <c r="E15" t="n">
+        <v>38</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3.7752</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>9</v>
+      </c>
+      <c r="M15" t="n">
+        <v>29</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="Q15" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S15" t="n">
+        <v>3</v>
+      </c>
+      <c r="V15" t="n">
         <v>1</v>
       </c>
-      <c r="Z14" t="n">
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>2026-08-17 11:58:22.184887</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-115818\20260817-115818.csv</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-115818\20260817-115818_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="D16" s="5">
+        <f>IFERROR(C16/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E16" t="n">
+        <v>11</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.9754</v>
+      </c>
+      <c r="G16" t="n">
         <v>4</v>
       </c>
-      <c r="AA14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t>13:31</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>5</v>
+      </c>
+      <c r="M16" t="n">
+        <v>6</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.4999999999999999</v>
+      </c>
+      <c r="S16" t="n">
+        <v>3</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1</v>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>2026-08-17 12:08:06.887277</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-120806\20260817-120806.csv</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-120806\20260817-120806_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Stage 2</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="9" t="n"/>
-      <c r="J15" s="9" t="n"/>
-      <c r="K15" s="9" t="n"/>
-      <c r="L15" s="9" t="n"/>
-      <c r="M15" s="9" t="n"/>
-      <c r="N15" s="9" t="n"/>
-      <c r="O15" s="9" t="n"/>
-      <c r="P15" s="9" t="n"/>
-      <c r="Q15" s="9" t="n"/>
-      <c r="R15" s="9" t="n"/>
-      <c r="S15" s="9" t="n"/>
-      <c r="T15" s="9" t="n"/>
-      <c r="U15" s="9" t="n"/>
-      <c r="V15" s="9" t="n"/>
-      <c r="W15" s="9" t="n"/>
-      <c r="X15" s="9" t="n"/>
-      <c r="Y15" s="9" t="n"/>
-      <c r="Z15" s="9" t="n"/>
-      <c r="AA15" s="9" t="n"/>
-      <c r="AB15" s="9" t="n"/>
-      <c r="AC15" s="9" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>stage2_threshold_staircase</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="5">
-        <f>IFERROR(S16/$B$5,"")</f>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="9" t="n"/>
+      <c r="L17" s="9" t="n"/>
+      <c r="M17" s="9" t="n"/>
+      <c r="N17" s="9" t="n"/>
+      <c r="O17" s="9" t="n"/>
+      <c r="P17" s="9" t="n"/>
+      <c r="Q17" s="9" t="n"/>
+      <c r="R17" s="9" t="n"/>
+      <c r="S17" s="9" t="n"/>
+      <c r="T17" s="9" t="n"/>
+      <c r="U17" s="9" t="n"/>
+      <c r="V17" s="9" t="n"/>
+      <c r="W17" s="9" t="n"/>
+      <c r="X17" s="9" t="n"/>
+      <c r="Y17" s="9" t="n"/>
+      <c r="Z17" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="D18" s="5">
+        <f>IFERROR(C18/$B$5,"")</f>
         <v/>
       </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr">
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y18" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135342\20260811-135342.csv</t>
-        </is>
-      </c>
-      <c r="Y16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>stage2_threshold_staircase</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>68</v>
-      </c>
-      <c r="D17" t="n">
-        <v>6.3955</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>40</v>
-      </c>
-      <c r="I17" t="n">
-        <v>28</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>7</v>
-      </c>
-      <c r="M17" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="N17" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="R17" t="b">
-        <v>0</v>
-      </c>
-      <c r="T17" s="5">
-        <f>IFERROR(S17/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>2026-08-11 13:51:34.028274</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135132\20260811-135132.csv</t>
-        </is>
-      </c>
-      <c r="Y17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>13:51</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>stage2_threshold_staircase</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>69</v>
-      </c>
-      <c r="D18" t="n">
-        <v>10.4654</v>
-      </c>
-      <c r="F18" t="n">
-        <v>9</v>
-      </c>
-      <c r="G18" t="n">
-        <v>26</v>
-      </c>
-      <c r="H18" t="n">
-        <v>29</v>
-      </c>
-      <c r="I18" t="n">
-        <v>14</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>7</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0.325</v>
-      </c>
-      <c r="R18" t="b">
-        <v>0</v>
-      </c>
-      <c r="T18" s="5">
-        <f>IFERROR(S18/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>2026-08-11 13:53:54.632954</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135354\20260811-135354.csv</t>
-        </is>
-      </c>
-      <c r="Y18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC18" t="inlineStr">
-        <is>
-          <t>13:53</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="D19" s="5">
+        <f>IFERROR(C19/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E19" t="n">
+        <v>68</v>
+      </c>
+      <c r="F19" t="n">
+        <v>6.3955</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>40</v>
+      </c>
+      <c r="M19" t="n">
+        <v>28</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>7</v>
+      </c>
+      <c r="P19" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="Q19" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="U19" t="b">
+        <v>0</v>
+      </c>
+      <c r="V19" t="n">
+        <v>1</v>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:51:34.028274</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135132\20260811-135132.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="D20" s="5">
+        <f>IFERROR(C20/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E20" t="n">
+        <v>69</v>
+      </c>
+      <c r="F20" t="n">
+        <v>10.4654</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>9</v>
+      </c>
+      <c r="K20" t="n">
+        <v>26</v>
+      </c>
+      <c r="L20" t="n">
+        <v>29</v>
+      </c>
+      <c r="M20" t="n">
+        <v>14</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>7</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="U20" t="b">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>1</v>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:53:54.632954</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135354\20260811-135354.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>stage2_threshold_staircase</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="D21" s="5">
+        <f>IFERROR(C21/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E21" t="n">
         <v>33</v>
       </c>
-      <c r="D19" t="n">
+      <c r="F21" t="n">
         <v>3.078</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G21" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" t="n">
         <v>7</v>
       </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
         <v>13</v>
       </c>
-      <c r="I19" t="n">
+      <c r="M21" t="n">
         <v>20</v>
       </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
         <v>7</v>
       </c>
-      <c r="M19" t="n">
+      <c r="P21" t="n">
         <v>10.5</v>
       </c>
-      <c r="N19" s="4" t="n">
+      <c r="Q21" s="4" t="n">
         <v>0.3</v>
       </c>
-      <c r="O19" t="n">
+      <c r="R21" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="T21" t="n">
         <v>0.6060606060606061</v>
       </c>
-      <c r="R19" t="b">
-        <v>0</v>
-      </c>
-      <c r="T19" s="5">
-        <f>IFERROR(S19/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="V19" t="inlineStr">
+      <c r="U21" t="b">
+        <v>0</v>
+      </c>
+      <c r="V21" t="n">
+        <v>1</v>
+      </c>
+      <c r="X21" t="inlineStr">
         <is>
           <t>2026-08-13 13:41:49.500571</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260813-134148\20260813-134148.csv</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
+      <c r="Z21" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260813-134148\20260813-134148_struct.mat</t>
-        </is>
-      </c>
-      <c r="Y19" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB19" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t>13:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Num. Sessions column shows a value only for an actual merge
Blank for an ordinary, un-merged row instead of a bare "1" -- a single
session isn't "combined," so a count there was misleading. Already sits
immediately before Notes (column V, Notes at W).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -742,9 +742,6 @@
       <c r="S9" t="n">
         <v>2</v>
       </c>
-      <c r="V9" t="n">
-        <v>1</v>
-      </c>
       <c r="W9" t="inlineStr">
         <is>
           <t>handled by hand</t>
@@ -815,9 +812,6 @@
       <c r="S10" t="n">
         <v>2</v>
       </c>
-      <c r="V10" t="n">
-        <v>1</v>
-      </c>
       <c r="X10" t="inlineStr">
         <is>
           <t>2026-08-11 13:46:30.773972</t>
@@ -889,9 +883,6 @@
       <c r="S11" t="n">
         <v>2</v>
       </c>
-      <c r="V11" t="n">
-        <v>1</v>
-      </c>
       <c r="X11" t="inlineStr">
         <is>
           <t>2026-08-13 11:14:02.776900</t>
@@ -944,9 +935,6 @@
       <c r="N12" t="n">
         <v>0</v>
       </c>
-      <c r="V12" t="n">
-        <v>1</v>
-      </c>
       <c r="X12" t="inlineStr">
         <is>
           <t>2026-08-13 13:22:19.337954</t>
@@ -1018,9 +1006,6 @@
       <c r="S13" t="n">
         <v>2</v>
       </c>
-      <c r="V13" t="n">
-        <v>1</v>
-      </c>
       <c r="X13" t="inlineStr">
         <is>
           <t>2026-08-13 13:29:35.160305</t>
@@ -1097,9 +1082,6 @@
       <c r="S14" t="n">
         <v>2</v>
       </c>
-      <c r="V14" t="n">
-        <v>1</v>
-      </c>
       <c r="X14" t="inlineStr">
         <is>
           <t>2026-08-13 13:31:59.325021</t>
@@ -1176,9 +1158,6 @@
       <c r="S15" t="n">
         <v>3</v>
       </c>
-      <c r="V15" t="n">
-        <v>1</v>
-      </c>
       <c r="X15" t="inlineStr">
         <is>
           <t>2026-08-17 11:58:22.184887</t>
@@ -1254,9 +1233,6 @@
       </c>
       <c r="S16" t="n">
         <v>3</v>
-      </c>
-      <c r="V16" t="n">
-        <v>1</v>
       </c>
       <c r="X16" t="inlineStr">
         <is>
@@ -1332,9 +1308,6 @@
       <c r="N18" t="n">
         <v>0</v>
       </c>
-      <c r="V18" t="n">
-        <v>1</v>
-      </c>
       <c r="Y18" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135342\20260811-135342.csv</t>
@@ -1398,9 +1371,6 @@
       <c r="U19" t="b">
         <v>0</v>
       </c>
-      <c r="V19" t="n">
-        <v>1</v>
-      </c>
       <c r="X19" t="inlineStr">
         <is>
           <t>2026-08-11 13:51:34.028274</t>
@@ -1469,9 +1439,6 @@
       <c r="U20" t="b">
         <v>0</v>
       </c>
-      <c r="V20" t="n">
-        <v>1</v>
-      </c>
       <c r="X20" t="inlineStr">
         <is>
           <t>2026-08-11 13:53:54.632954</t>
@@ -1545,9 +1512,6 @@
       </c>
       <c r="U21" t="b">
         <v>0</v>
-      </c>
-      <c r="V21" t="n">
-        <v>1</v>
       </c>
       <c r="X21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix stale hidden-column flag; merge the test subject like any other
ws.column_dimensions is keyed by letter and survives row deletes -- once
'Session started' had sat at a given letter in an earlier schema
iteration, that letter's hidden=True flag lingered forever even after the
column moved elsewhere, which is why Num. Sessions showed up hidden. Now
every column's hidden flag is reset before re-hiding only the current
Session started column.

Also removed the test-subject merge exclusion entirely, per explicit
instruction -- bench-test sessions now merge exactly like a real animal's
would, no more toggling a debug flag back and forth to verify it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z21"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="14"/>
@@ -471,7 +471,7 @@
     <col customWidth="1" max="19" min="19" width="14"/>
     <col customWidth="1" max="20" min="20" width="14"/>
     <col customWidth="1" max="21" min="21" width="14"/>
-    <col customWidth="1" hidden="1" max="22" min="22" width="14"/>
+    <col customWidth="1" max="22" min="22" width="14"/>
     <col customWidth="1" max="23" min="23" width="14"/>
     <col customWidth="1" hidden="1" max="24" min="24" width="14"/>
     <col customWidth="1" max="25" min="25" width="14"/>
@@ -704,10 +704,10 @@
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>15</v>
+        <v>140</v>
       </c>
       <c r="F9" t="n">
-        <v>8.220500000000001</v>
+        <v>18.6963</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -716,13 +716,13 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>6</v>
+        <v>101</v>
       </c>
       <c r="M9" t="n">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -742,6 +742,9 @@
       <c r="S9" t="n">
         <v>2</v>
       </c>
+      <c r="V9" t="n">
+        <v>2</v>
+      </c>
       <c r="W9" t="inlineStr">
         <is>
           <t>handled by hand</t>
@@ -749,24 +752,29 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-08-11 13:41:46.605630</t>
+          <t>2026-08-11 13:41:46.605630; 2026-08-11 13:46:30.773972</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134145\20260811-134145.csv</t>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134145\20260811-134145.csv; C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134630\20260811-134630.csv</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134145\20260811-134145_combined_struct.mat</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13:46</t>
+          <t>11:14</t>
         </is>
       </c>
       <c r="D10" s="5">
@@ -774,10 +782,16 @@
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
-        <v>10.4758</v>
+        <v>4.019900000000001</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -786,40 +800,45 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>7</v>
+        <v>1.75</v>
       </c>
       <c r="P10" t="n">
-        <v>7</v>
+        <v>1.75</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="R10" t="n">
-        <v>0.5</v>
+        <v>0.4999999999999999</v>
       </c>
       <c r="S10" t="n">
         <v>2</v>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-08-11 13:46:30.773972</t>
+          <t>2026-08-13 11:14:02.776900</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260811-134630\20260811-134630.csv</t>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-111402\20260813-111402.csv</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-111402\20260813-111402_struct.mat</t>
         </is>
       </c>
     </row>
@@ -831,7 +850,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11:14</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="D11" s="5">
@@ -839,15 +858,6 @@
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
-      </c>
-      <c r="F11" t="n">
-        <v>4.019900000000001</v>
-      </c>
-      <c r="G11" t="n">
-        <v>4</v>
-      </c>
-      <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
@@ -860,42 +870,22 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
-      <c r="O11" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="P11" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="Q11" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0.4999999999999999</v>
-      </c>
-      <c r="S11" t="n">
-        <v>2</v>
-      </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-08-13 11:14:02.776900</t>
+          <t>2026-08-13 13:22:19.337954</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-111402\20260813-111402.csv</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-111402\20260813-111402_struct.mat</t>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132218\20260813-132218.csv</t>
         </is>
       </c>
     </row>
@@ -907,7 +897,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:29</t>
         </is>
       </c>
       <c r="D12" s="5">
@@ -915,46 +905,78 @@
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>47</v>
+      </c>
+      <c r="F12" t="n">
+        <v>11.9186</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>12</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S12" t="n">
+        <v>2</v>
+      </c>
+      <c r="V12" t="n">
+        <v>2</v>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-08-13 13:22:19.337954</t>
+          <t>2026-08-13 13:29:35.160305; 2026-08-13 13:31:59.325021</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132218\20260813-132218.csv</t>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132934\20260813-132934.csv; C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-133158\20260813-133158.csv</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132934\20260813-132934_combined_struct.mat</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>13:29</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="D13" s="5">
@@ -962,34 +984,34 @@
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="F13" t="n">
-        <v>10.3488</v>
+        <v>5.7506</v>
       </c>
       <c r="G13" t="n">
         <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="M13" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="N13" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
         <v>1.75</v>
@@ -1001,128 +1023,70 @@
         <v>0.05</v>
       </c>
       <c r="R13" t="n">
-        <v>0.5</v>
+        <v>0.4999999999999999</v>
       </c>
       <c r="S13" t="n">
+        <v>3</v>
+      </c>
+      <c r="V13" t="n">
         <v>2</v>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-08-13 13:29:35.160305</t>
+          <t>2026-08-17 11:58:22.184887; 2026-08-17 12:08:06.887277</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132934\20260813-132934.csv</t>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-115818\20260817-115818.csv; C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-120806\20260817-120806.csv</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-132934\20260813-132934_struct.mat</t>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-115818\20260817-115818_combined_struct.mat</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>13:31</t>
-        </is>
-      </c>
-      <c r="D14" s="5">
-        <f>IFERROR(C14/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="E14" t="n">
-        <v>15</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1.5698</v>
-      </c>
-      <c r="G14" t="n">
-        <v>4</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>7</v>
-      </c>
-      <c r="M14" t="n">
-        <v>8</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="P14" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="S14" t="n">
-        <v>2</v>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>2026-08-13 13:31:59.325021</t>
-        </is>
-      </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-133158\20260813-133158.csv</t>
-        </is>
-      </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260813-133158\20260813-133158_struct.mat</t>
-        </is>
-      </c>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="9" t="n"/>
+      <c r="J14" s="9" t="n"/>
+      <c r="K14" s="9" t="n"/>
+      <c r="L14" s="9" t="n"/>
+      <c r="M14" s="9" t="n"/>
+      <c r="N14" s="9" t="n"/>
+      <c r="O14" s="9" t="n"/>
+      <c r="P14" s="9" t="n"/>
+      <c r="Q14" s="9" t="n"/>
+      <c r="R14" s="9" t="n"/>
+      <c r="S14" s="9" t="n"/>
+      <c r="T14" s="9" t="n"/>
+      <c r="U14" s="9" t="n"/>
+      <c r="V14" s="9" t="n"/>
+      <c r="W14" s="9" t="n"/>
+      <c r="X14" s="9" t="n"/>
+      <c r="Y14" s="9" t="n"/>
+      <c r="Z14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>11:58</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
       <c r="D15" s="5">
         <f>IFERROR(C15/$B$5,"")</f>
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>38</v>
-      </c>
-      <c r="F15" t="n">
-        <v>3.7752</v>
-      </c>
-      <c r="G15" t="n">
-        <v>4</v>
-      </c>
-      <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
@@ -1135,54 +1099,30 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
-      <c r="O15" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="P15" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="Q15" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="S15" t="n">
-        <v>3</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>2026-08-17 11:58:22.184887</t>
-        </is>
-      </c>
+      <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-115818\20260817-115818.csv</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-115818\20260817-115818_struct.mat</t>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135342\20260811-135342.csv</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="D16" s="5">
@@ -1190,340 +1130,140 @@
         <v/>
       </c>
       <c r="E16" t="n">
-        <v>11</v>
+        <v>137</v>
       </c>
       <c r="F16" t="n">
-        <v>1.9754</v>
-      </c>
-      <c r="G16" t="n">
+        <v>16.8609</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>9</v>
+      </c>
+      <c r="K16" t="n">
+        <v>26</v>
+      </c>
+      <c r="L16" t="n">
+        <v>69</v>
+      </c>
+      <c r="M16" t="n">
+        <v>42</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>7</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="U16" t="b">
+        <v>0</v>
+      </c>
+      <c r="V16" t="n">
+        <v>2</v>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>2026-08-11 13:51:34.028274; 2026-08-11 13:53:54.632954</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135132\20260811-135132.csv; C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135354\20260811-135354.csv</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135132\20260811-135132_combined_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="D17" s="5">
+        <f>IFERROR(C17/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E17" t="n">
+        <v>33</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3.078</v>
+      </c>
+      <c r="G17" t="n">
         <v>4</v>
       </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
         <v>5</v>
       </c>
-      <c r="M16" t="n">
-        <v>6</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="P16" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="Q16" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0.4999999999999999</v>
-      </c>
-      <c r="S16" t="n">
-        <v>3</v>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>2026-08-17 12:08:06.887277</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-120806\20260817-120806.csv</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage1\sessions\20260817-120806\20260817-120806_struct.mat</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Stage 2</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="9" t="n"/>
-      <c r="H17" s="9" t="n"/>
-      <c r="I17" s="9" t="n"/>
-      <c r="J17" s="9" t="n"/>
-      <c r="K17" s="9" t="n"/>
-      <c r="L17" s="9" t="n"/>
-      <c r="M17" s="9" t="n"/>
-      <c r="N17" s="9" t="n"/>
-      <c r="O17" s="9" t="n"/>
-      <c r="P17" s="9" t="n"/>
-      <c r="Q17" s="9" t="n"/>
-      <c r="R17" s="9" t="n"/>
-      <c r="S17" s="9" t="n"/>
-      <c r="T17" s="9" t="n"/>
-      <c r="U17" s="9" t="n"/>
-      <c r="V17" s="9" t="n"/>
-      <c r="W17" s="9" t="n"/>
-      <c r="X17" s="9" t="n"/>
-      <c r="Y17" s="9" t="n"/>
-      <c r="Z17" s="9" t="n"/>
-    </row>
-    <row r="18">
-      <c r="D18" s="5">
-        <f>IFERROR(C18/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135342\20260811-135342.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>13:51</t>
-        </is>
-      </c>
-      <c r="D19" s="5">
-        <f>IFERROR(C19/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="E19" t="n">
-        <v>68</v>
-      </c>
-      <c r="F19" t="n">
-        <v>6.3955</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
-        <v>40</v>
-      </c>
-      <c r="M19" t="n">
-        <v>28</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="n">
+      <c r="J17" t="n">
         <v>7</v>
       </c>
-      <c r="P19" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="Q19" s="4" t="n">
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>13</v>
+      </c>
+      <c r="M17" t="n">
+        <v>20</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>7</v>
+      </c>
+      <c r="P17" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="Q17" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="R17" t="n">
         <v>0.5</v>
       </c>
-      <c r="R19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="T19" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="U19" t="b">
-        <v>0</v>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>2026-08-11 13:51:34.028274</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135132\20260811-135132.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>13:53</t>
-        </is>
-      </c>
-      <c r="D20" s="5">
-        <f>IFERROR(C20/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="E20" t="n">
-        <v>69</v>
-      </c>
-      <c r="F20" t="n">
-        <v>10.4654</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="n">
-        <v>9</v>
-      </c>
-      <c r="K20" t="n">
-        <v>26</v>
-      </c>
-      <c r="L20" t="n">
-        <v>29</v>
-      </c>
-      <c r="M20" t="n">
-        <v>14</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="n">
-        <v>7</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0.325</v>
-      </c>
-      <c r="U20" t="b">
-        <v>0</v>
-      </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>2026-08-11 13:53:54.632954</t>
-        </is>
-      </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260811-135354\20260811-135354.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>13:41</t>
-        </is>
-      </c>
-      <c r="D21" s="5">
-        <f>IFERROR(C21/$B$5,"")</f>
-        <v/>
-      </c>
-      <c r="E21" t="n">
-        <v>33</v>
-      </c>
-      <c r="F21" t="n">
-        <v>3.078</v>
-      </c>
-      <c r="G21" t="n">
-        <v>4</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>5</v>
-      </c>
-      <c r="J21" t="n">
-        <v>7</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
-        <v>13</v>
-      </c>
-      <c r="M21" t="n">
-        <v>20</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="n">
-        <v>7</v>
-      </c>
-      <c r="P21" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="Q21" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="T21" t="n">
+      <c r="T17" t="n">
         <v>0.6060606060606061</v>
       </c>
-      <c r="U21" t="b">
-        <v>0</v>
-      </c>
-      <c r="X21" t="inlineStr">
+      <c r="U17" t="b">
+        <v>0</v>
+      </c>
+      <c r="X17" t="inlineStr">
         <is>
           <t>2026-08-13 13:41:49.500571</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260813-134148\20260813-134148.csv</t>
         </is>
       </c>
-      <c r="Z21" t="inlineStr">
+      <c r="Z17" t="inlineStr">
         <is>
           <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260813-134148\20260813-134148_struct.mat</t>
         </is>

</xml_diff>

<commit_message>
Update training_log.xlsx from DESKTOP-MN31N9D
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="14"/>
@@ -1269,6 +1269,88 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="D18" s="5">
+        <f>IFERROR(C18/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E18" t="n">
+        <v>29</v>
+      </c>
+      <c r="F18" t="n">
+        <v>7.306100000000001</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>20</v>
+      </c>
+      <c r="M18" t="n">
+        <v>9</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="P18" t="n">
+        <v>5.250000000000001</v>
+      </c>
+      <c r="Q18" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="U18" t="b">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>2</v>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>2026-08-17 13:21:11.675718; 2026-08-17 13:22:19.871948</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260817-132110\20260817-132110.csv; C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260817-132219\20260817-132219.csv</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>C:\Users\2P-Behav\Documents\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Training\setups\Stage2\sessions\20260817-132110\20260817-132110_combined_struct.mat</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>